<commit_message>
expanded cook county data, still working on search sentiment
</commit_message>
<xml_diff>
--- a/phase_2/combined_CC_v5.xlsx
+++ b/phase_2/combined_CC_v5.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/daisyzhang/PF_research/phase_2/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:9_{C4F39358-1B35-044B-8CDC-0B775B6E682C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0263B4BF-39E5-F144-BE42-8C8360E60413}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1080" yWindow="1240" windowWidth="16480" windowHeight="16300" xr2:uid="{10C483BF-6D09-AE42-8B7E-3DBCF72AD855}"/>
+    <workbookView xWindow="14660" yWindow="740" windowWidth="14740" windowHeight="16300" xr2:uid="{10C483BF-6D09-AE42-8B7E-3DBCF72AD855}"/>
   </bookViews>
   <sheets>
     <sheet name="combined_CC_v5" sheetId="1" r:id="rId1"/>
@@ -57,7 +57,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="1">
-    <numFmt numFmtId="165" formatCode="0.0"/>
+    <numFmt numFmtId="164" formatCode="0.0"/>
   </numFmts>
   <fonts count="22" x14ac:knownFonts="1">
     <font>
@@ -402,7 +402,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="10">
+  <borders count="11">
     <border>
       <left/>
       <right/>
@@ -517,6 +517,21 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="42">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
@@ -562,14 +577,16 @@
     <xf numFmtId="0" fontId="1" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="22" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="19" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="20" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="21" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="4" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="4" fontId="0" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="42">
     <cellStyle name="20% - Accent1" xfId="19" builtinId="30" customBuiltin="1"/>
@@ -949,6 +966,7 @@
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="19.83203125" customWidth="1"/>
+    <col min="6" max="6" width="15.83203125" customWidth="1"/>
     <col min="10" max="10" width="22.1640625" customWidth="1"/>
   </cols>
   <sheetData>
@@ -1001,7 +1019,7 @@
         <v>0</v>
       </c>
       <c r="F2">
-        <v>27606708.140000001</v>
+        <v>28859652.989999998</v>
       </c>
       <c r="G2">
         <v>39461715</v>
@@ -1030,7 +1048,7 @@
         <v>0</v>
       </c>
       <c r="F3">
-        <v>29775106.309999999</v>
+        <v>28628423.140000001</v>
       </c>
       <c r="G3">
         <v>38516587</v>
@@ -1062,7 +1080,7 @@
         <v>0</v>
       </c>
       <c r="F4">
-        <v>30069627.420000002</v>
+        <v>34437875.060000002</v>
       </c>
       <c r="G4">
         <v>44908188</v>
@@ -1094,7 +1112,7 @@
         <v>0</v>
       </c>
       <c r="F5">
-        <v>28240772.579999998</v>
+        <v>23660620.289999999</v>
       </c>
       <c r="G5">
         <v>43186487</v>
@@ -1126,7 +1144,7 @@
         <v>65</v>
       </c>
       <c r="F6">
-        <v>29078637.809999999</v>
+        <v>23554200.48</v>
       </c>
       <c r="G6">
         <v>44674213</v>
@@ -1158,7 +1176,7 @@
         <v>125</v>
       </c>
       <c r="F7">
-        <v>30145865.18</v>
+        <v>28153259.559999999</v>
       </c>
       <c r="G7">
         <v>43941538</v>
@@ -1190,7 +1208,7 @@
         <v>222</v>
       </c>
       <c r="F8">
-        <v>28859652.989999998</v>
+        <v>27798957.960000001</v>
       </c>
       <c r="G8">
         <v>44380916</v>
@@ -1222,7 +1240,7 @@
         <v>206</v>
       </c>
       <c r="F9">
-        <v>28628423.140000001</v>
+        <v>29768756.100000001</v>
       </c>
       <c r="G9">
         <v>43470075</v>
@@ -1254,7 +1272,7 @@
         <v>145</v>
       </c>
       <c r="F10">
-        <v>34437875.060000002</v>
+        <v>31635672.07</v>
       </c>
       <c r="G10">
         <v>45070349</v>
@@ -1286,7 +1304,7 @@
         <v>9</v>
       </c>
       <c r="F11">
-        <v>23660620.289999999</v>
+        <v>29923428.440000001</v>
       </c>
       <c r="G11">
         <v>47721320</v>
@@ -1318,7 +1336,7 @@
         <v>0</v>
       </c>
       <c r="F12">
-        <v>23554200.48</v>
+        <v>30204767.940000001</v>
       </c>
       <c r="G12">
         <v>41599867</v>
@@ -1350,7 +1368,7 @@
         <v>0</v>
       </c>
       <c r="F13">
-        <v>28153259.559999999</v>
+        <v>30119564.300000001</v>
       </c>
       <c r="G13">
         <v>39316959</v>
@@ -1382,7 +1400,7 @@
         <v>0</v>
       </c>
       <c r="F14">
-        <v>27798957.960000001</v>
+        <v>29838990.109999999</v>
       </c>
       <c r="G14">
         <v>39925460</v>
@@ -1414,7 +1432,7 @@
         <v>0</v>
       </c>
       <c r="F15">
-        <v>29768756.100000001</v>
+        <v>28282114.559999999</v>
       </c>
       <c r="G15">
         <v>38776369</v>
@@ -1446,7 +1464,7 @@
         <v>0</v>
       </c>
       <c r="F16">
-        <v>31635672.07</v>
+        <v>35403923.460000001</v>
       </c>
       <c r="G16">
         <v>43039648</v>
@@ -1478,7 +1496,7 @@
         <v>0</v>
       </c>
       <c r="F17">
-        <v>29923428.440000001</v>
+        <v>53375007.520000003</v>
       </c>
       <c r="G17">
         <v>41725144</v>
@@ -1510,7 +1528,7 @@
         <v>47</v>
       </c>
       <c r="F18">
-        <v>30204767.940000001</v>
+        <v>56260939.890000001</v>
       </c>
       <c r="G18">
         <v>42713453</v>
@@ -1542,7 +1560,7 @@
         <v>207</v>
       </c>
       <c r="F19">
-        <v>30119564.300000001</v>
+        <v>65962180.950000003</v>
       </c>
       <c r="G19">
         <v>42230444</v>
@@ -1574,7 +1592,7 @@
         <v>303</v>
       </c>
       <c r="F20">
-        <v>29838990.109999999</v>
+        <v>62493840.670000002</v>
       </c>
       <c r="G20">
         <v>41696808</v>
@@ -1606,7 +1624,7 @@
         <v>322</v>
       </c>
       <c r="F21">
-        <v>28282114.559999999</v>
+        <v>69627843.680000007</v>
       </c>
       <c r="G21">
         <v>41446797</v>
@@ -1638,7 +1656,7 @@
         <v>153</v>
       </c>
       <c r="F22">
-        <v>35403923.460000001</v>
+        <v>75197274.150000006</v>
       </c>
       <c r="G22">
         <v>43060220</v>
@@ -1670,7 +1688,7 @@
         <v>18</v>
       </c>
       <c r="F23">
-        <v>53375007.520000003</v>
+        <v>69006512.349999994</v>
       </c>
       <c r="G23">
         <v>45583905</v>
@@ -1702,7 +1720,7 @@
         <v>0</v>
       </c>
       <c r="F24">
-        <v>56260939.890000001</v>
+        <v>68263674.450000003</v>
       </c>
       <c r="G24">
         <v>40504644</v>
@@ -1734,7 +1752,7 @@
         <v>0</v>
       </c>
       <c r="F25">
-        <v>65962180.950000003</v>
+        <v>69553963.390000001</v>
       </c>
       <c r="G25">
         <v>36391192</v>
@@ -1766,7 +1784,7 @@
         <v>0</v>
       </c>
       <c r="F26">
-        <v>62493840.670000002</v>
+        <v>67405675.010000005</v>
       </c>
       <c r="G26">
         <v>37786715</v>
@@ -1798,7 +1816,7 @@
         <v>0</v>
       </c>
       <c r="F27">
-        <v>69627843.680000007</v>
+        <v>67825677.280000001</v>
       </c>
       <c r="G27">
         <v>37488628</v>
@@ -1830,7 +1848,7 @@
         <v>0</v>
       </c>
       <c r="F28">
-        <v>75197274.150000006</v>
+        <v>81531774.900000006</v>
       </c>
       <c r="G28">
         <v>41072863</v>
@@ -1862,7 +1880,7 @@
         <v>5</v>
       </c>
       <c r="F29">
-        <v>69006512.349999994</v>
+        <v>56297195.439999998</v>
       </c>
       <c r="G29">
         <v>39786074</v>
@@ -1894,7 +1912,7 @@
         <v>30</v>
       </c>
       <c r="F30">
-        <v>68263674.450000003</v>
+        <v>56233617.770000003</v>
       </c>
       <c r="G30">
         <v>41178701</v>
@@ -1926,7 +1944,7 @@
         <v>202</v>
       </c>
       <c r="F31">
-        <v>69553963.390000001</v>
+        <v>66386157.289999999</v>
       </c>
       <c r="G31">
         <v>41193119</v>
@@ -1958,7 +1976,7 @@
         <v>264</v>
       </c>
       <c r="F32">
-        <v>67405675.010000005</v>
+        <v>65212635.32</v>
       </c>
       <c r="G32">
         <v>39969663</v>
@@ -1990,7 +2008,7 @@
         <v>170</v>
       </c>
       <c r="F33">
-        <v>67825677.280000001</v>
+        <v>69421573.859999999</v>
       </c>
       <c r="G33">
         <v>41021524</v>
@@ -2022,7 +2040,7 @@
         <v>124</v>
       </c>
       <c r="F34">
-        <v>81531774.900000006</v>
+        <v>73119893.780000001</v>
       </c>
       <c r="G34">
         <v>42285990</v>
@@ -2054,7 +2072,7 @@
         <v>18</v>
       </c>
       <c r="F35">
-        <v>56297195.439999998</v>
+        <v>67781079.359999999</v>
       </c>
       <c r="G35">
         <v>43816126</v>
@@ -2086,7 +2104,7 @@
         <v>0</v>
       </c>
       <c r="F36">
-        <v>56233617.770000003</v>
+        <v>68994675.099999994</v>
       </c>
       <c r="G36">
         <v>38845428</v>
@@ -2118,7 +2136,7 @@
         <v>0</v>
       </c>
       <c r="F37">
-        <v>66386157.289999999</v>
+        <v>68813719.370000005</v>
       </c>
       <c r="G37">
         <v>36051520</v>
@@ -2150,7 +2168,7 @@
         <v>0</v>
       </c>
       <c r="F38">
-        <v>65212635.32</v>
+        <v>67466235.420000002</v>
       </c>
       <c r="G38">
         <v>35994884</v>
@@ -2182,7 +2200,7 @@
         <v>0</v>
       </c>
       <c r="F39">
-        <v>69421573.859999999</v>
+        <v>68308547.760000005</v>
       </c>
       <c r="G39">
         <v>35402320</v>
@@ -2214,7 +2232,7 @@
         <v>0</v>
       </c>
       <c r="F40">
-        <v>73119893.780000001</v>
+        <v>81326655.430000007</v>
       </c>
       <c r="G40">
         <v>39893267</v>
@@ -2246,7 +2264,7 @@
         <v>0</v>
       </c>
       <c r="F41">
-        <v>67781079.359999999</v>
+        <v>58821645.289999999</v>
       </c>
       <c r="G41">
         <v>39373551</v>
@@ -2278,7 +2296,7 @@
         <v>128</v>
       </c>
       <c r="F42">
-        <v>68994675.099999994</v>
+        <v>56928622.950000003</v>
       </c>
       <c r="G42">
         <v>40431897</v>
@@ -2310,7 +2328,7 @@
         <v>187</v>
       </c>
       <c r="F43">
-        <v>68813719.370000005</v>
+        <v>69006437.459999993</v>
       </c>
       <c r="G43">
         <v>39599893</v>
@@ -2342,7 +2360,7 @@
         <v>291</v>
       </c>
       <c r="F44">
-        <v>67466235.420000002</v>
+        <v>65512498.039999999</v>
       </c>
       <c r="G44">
         <v>39465213</v>
@@ -2374,7 +2392,7 @@
         <v>304</v>
       </c>
       <c r="F45">
-        <v>68308547.760000005</v>
+        <v>74052335.969999999</v>
       </c>
       <c r="G45">
         <v>40048581</v>
@@ -2406,7 +2424,7 @@
         <v>125</v>
       </c>
       <c r="F46">
-        <v>81326655.430000007</v>
+        <v>76306913.900000006</v>
       </c>
       <c r="G46">
         <v>41597367</v>
@@ -2438,7 +2456,7 @@
         <v>0</v>
       </c>
       <c r="F47">
-        <v>58821645.289999999</v>
+        <v>70785493.510000005</v>
       </c>
       <c r="G47">
         <v>43590423</v>
@@ -2470,7 +2488,7 @@
         <v>0</v>
       </c>
       <c r="F48">
-        <v>56928622.950000003</v>
+        <v>73166741.219999999</v>
       </c>
       <c r="G48">
         <v>37544425</v>
@@ -2502,7 +2520,7 @@
         <v>0</v>
       </c>
       <c r="F49">
-        <v>69006437.459999993</v>
+        <v>70562415.079999998</v>
       </c>
       <c r="G49">
         <v>35501409</v>
@@ -2534,7 +2552,7 @@
         <v>0</v>
       </c>
       <c r="F50">
-        <v>65512498.039999999</v>
+        <v>71626171.019999996</v>
       </c>
       <c r="G50">
         <v>33033146</v>
@@ -2566,7 +2584,7 @@
         <v>0</v>
       </c>
       <c r="F51">
-        <v>74052335.969999999</v>
+        <v>69887841.409999996</v>
       </c>
       <c r="G51">
         <v>34944862</v>
@@ -2598,7 +2616,7 @@
         <v>0</v>
       </c>
       <c r="F52">
-        <v>76306913.900000006</v>
+        <v>80402424.640000001</v>
       </c>
       <c r="G52">
         <v>31161797</v>
@@ -2630,7 +2648,7 @@
         <v>0</v>
       </c>
       <c r="F53">
-        <v>70785493.510000005</v>
+        <v>54919556.82</v>
       </c>
       <c r="G53">
         <v>37874004</v>
@@ -2662,7 +2680,7 @@
         <v>33</v>
       </c>
       <c r="F54">
-        <v>73166741.219999999</v>
+        <v>56461598.159999996</v>
       </c>
       <c r="G54">
         <v>39701953</v>
@@ -2694,7 +2712,7 @@
         <v>127</v>
       </c>
       <c r="F55">
-        <v>70562415.079999998</v>
+        <v>68656689.25</v>
       </c>
       <c r="G55">
         <v>39583408</v>
@@ -2726,7 +2744,7 @@
         <v>350</v>
       </c>
       <c r="F56">
-        <v>71626171.019999996</v>
+        <v>67846113.5</v>
       </c>
       <c r="G56">
         <v>38544689</v>
@@ -2758,7 +2776,7 @@
         <v>222</v>
       </c>
       <c r="F57">
-        <v>69887841.409999996</v>
+        <v>73986096.510000005</v>
       </c>
       <c r="G57">
         <v>39332880</v>
@@ -2790,7 +2808,7 @@
         <v>142</v>
       </c>
       <c r="F58">
-        <v>80402424.640000001</v>
+        <v>75961708.730000004</v>
       </c>
       <c r="G58">
         <v>40504073</v>
@@ -2822,7 +2840,7 @@
         <v>0</v>
       </c>
       <c r="F59">
-        <v>54919556.82</v>
+        <v>72537143.530000001</v>
       </c>
       <c r="G59">
         <v>41748713</v>
@@ -2854,7 +2872,7 @@
         <v>0</v>
       </c>
       <c r="F60">
-        <v>56461598.159999996</v>
+        <v>73233944.890000001</v>
       </c>
       <c r="G60">
         <v>36961008</v>
@@ -2886,7 +2904,7 @@
         <v>0</v>
       </c>
       <c r="F61">
-        <v>68656689.25</v>
+        <v>71052949.489999995</v>
       </c>
       <c r="G61">
         <v>34808947</v>
@@ -2918,7 +2936,7 @@
         <v>0</v>
       </c>
       <c r="F62">
-        <v>67846113.5</v>
+        <v>72032875.239999995</v>
       </c>
       <c r="G62">
         <v>36072142</v>
@@ -2950,7 +2968,7 @@
         <v>0</v>
       </c>
       <c r="F63">
-        <v>73986096.510000005</v>
+        <v>69939707.75</v>
       </c>
       <c r="G63">
         <v>34858049</v>
@@ -2982,7 +3000,7 @@
         <v>0</v>
       </c>
       <c r="F64">
-        <v>75961708.730000004</v>
+        <v>81607813.209999993</v>
       </c>
       <c r="G64">
         <v>23233727</v>
@@ -3014,7 +3032,7 @@
         <v>0</v>
       </c>
       <c r="F65">
-        <v>72537143.530000001</v>
+        <v>58933107.670000002</v>
       </c>
       <c r="G65">
         <v>8062778</v>
@@ -3046,7 +3064,7 @@
         <v>36</v>
       </c>
       <c r="F66">
-        <v>73233944.890000001</v>
+        <v>54947219.990000002</v>
       </c>
       <c r="G66">
         <v>9178429</v>
@@ -3078,7 +3096,7 @@
         <v>221</v>
       </c>
       <c r="F67">
-        <v>71052949.489999995</v>
+        <v>50419580.68</v>
       </c>
       <c r="G67">
         <v>10225049</v>
@@ -3110,7 +3128,7 @@
         <v>360</v>
       </c>
       <c r="F68">
-        <v>72032875.239999995</v>
+        <v>38476836.899999999</v>
       </c>
       <c r="G68">
         <v>12746594</v>
@@ -3158,7 +3176,7 @@
         <v>270</v>
       </c>
       <c r="F69">
-        <v>69939707.75</v>
+        <v>46109877.149999999</v>
       </c>
       <c r="G69">
         <v>12984554</v>
@@ -3206,7 +3224,7 @@
         <v>61</v>
       </c>
       <c r="F70">
-        <v>81607813.209999993</v>
+        <v>56464654.479999997</v>
       </c>
       <c r="G70">
         <v>13053733</v>
@@ -3254,7 +3272,7 @@
         <v>0</v>
       </c>
       <c r="F71">
-        <v>58933107.670000002</v>
+        <v>61177461.539999999</v>
       </c>
       <c r="G71">
         <v>13609917</v>
@@ -3302,7 +3320,7 @@
         <v>0</v>
       </c>
       <c r="F72">
-        <v>54947219.990000002</v>
+        <v>60080433.439999998</v>
       </c>
       <c r="G72">
         <v>11427941</v>
@@ -3350,7 +3368,7 @@
         <v>0</v>
       </c>
       <c r="F73">
-        <v>50419580.68</v>
+        <v>61922896.299999997</v>
       </c>
       <c r="G73">
         <v>11024833</v>
@@ -3382,7 +3400,7 @@
         <v>0</v>
       </c>
       <c r="F74">
-        <v>38476836.899999999</v>
+        <v>59972884.82</v>
       </c>
       <c r="G74">
         <v>10980903</v>
@@ -3414,7 +3432,7 @@
         <v>0</v>
       </c>
       <c r="F75">
-        <v>46109877.149999999</v>
+        <v>55502405.689999998</v>
       </c>
       <c r="G75">
         <v>10552678</v>
@@ -3446,7 +3464,7 @@
         <v>0</v>
       </c>
       <c r="F76">
-        <v>56464654.479999997</v>
+        <v>68824077.959999993</v>
       </c>
       <c r="G76">
         <v>13465695</v>
@@ -3478,7 +3496,7 @@
         <v>0</v>
       </c>
       <c r="F77">
-        <v>61177461.539999999</v>
+        <v>57567755.399999999</v>
       </c>
       <c r="G77">
         <v>13768950</v>
@@ -3510,7 +3528,7 @@
         <v>42</v>
       </c>
       <c r="F78">
-        <v>60080433.439999998</v>
+        <v>54773167.329999998</v>
       </c>
       <c r="G78">
         <v>15100909</v>
@@ -3542,7 +3560,7 @@
         <v>249</v>
       </c>
       <c r="F79">
-        <v>61922896.299999997</v>
+        <v>81000519.719999999</v>
       </c>
       <c r="G79">
         <v>16504335</v>
@@ -3573,8 +3591,8 @@
       <c r="E80">
         <v>264</v>
       </c>
-      <c r="F80">
-        <v>59972884.82</v>
+      <c r="F80" s="7">
+        <v>38476836.899999999</v>
       </c>
       <c r="G80">
         <v>18566992</v>
@@ -3605,8 +3623,8 @@
       <c r="E81">
         <v>333</v>
       </c>
-      <c r="F81">
-        <v>55502405.689999998</v>
+      <c r="F81" s="7">
+        <v>46109877.149999999</v>
       </c>
       <c r="G81">
         <v>19095700</v>
@@ -3637,8 +3655,8 @@
       <c r="E82">
         <v>148</v>
       </c>
-      <c r="F82">
-        <v>68824077.959999993</v>
+      <c r="F82" s="7">
+        <v>56464654.479999997</v>
       </c>
       <c r="G82">
         <v>20883918</v>
@@ -3669,8 +3687,8 @@
       <c r="E83">
         <v>31</v>
       </c>
-      <c r="F83">
-        <v>57567755.399999999</v>
+      <c r="F83" s="7">
+        <v>61177461.539999999</v>
       </c>
       <c r="G83">
         <v>21270174</v>
@@ -3701,8 +3719,8 @@
       <c r="E84">
         <v>0</v>
       </c>
-      <c r="F84">
-        <v>54773167.329999998</v>
+      <c r="F84" s="7">
+        <v>60080433.439999998</v>
       </c>
       <c r="G84">
         <v>18767083</v>
@@ -3733,8 +3751,8 @@
       <c r="E85">
         <v>0</v>
       </c>
-      <c r="F85">
-        <v>81000519.719999999</v>
+      <c r="F85" s="7">
+        <v>61922896.299999997</v>
       </c>
       <c r="G85">
         <v>17322199</v>
@@ -3765,6 +3783,12 @@
       <c r="E86">
         <v>0</v>
       </c>
+      <c r="F86" s="7">
+        <v>59972884.82</v>
+      </c>
+      <c r="G86">
+        <v>14367405</v>
+      </c>
     </row>
     <row r="87" spans="1:10" ht="18" x14ac:dyDescent="0.2">
       <c r="A87" s="1">
@@ -3782,6 +3806,12 @@
       <c r="E87">
         <v>0</v>
       </c>
+      <c r="F87" s="7">
+        <v>55502405.689999998</v>
+      </c>
+      <c r="G87">
+        <v>16409515</v>
+      </c>
     </row>
     <row r="88" spans="1:10" ht="18" x14ac:dyDescent="0.2">
       <c r="A88" s="1">
@@ -3799,6 +3829,12 @@
       <c r="E88">
         <v>0</v>
       </c>
+      <c r="F88" s="7">
+        <v>68824077.959999993</v>
+      </c>
+      <c r="G88">
+        <v>20245968</v>
+      </c>
     </row>
     <row r="89" spans="1:10" ht="18" x14ac:dyDescent="0.2">
       <c r="A89" s="1">
@@ -3816,6 +3852,12 @@
       <c r="E89">
         <v>0</v>
       </c>
+      <c r="F89" s="7">
+        <v>57567755.399999999</v>
+      </c>
+      <c r="G89">
+        <v>19866149</v>
+      </c>
     </row>
     <row r="90" spans="1:10" ht="18" x14ac:dyDescent="0.2">
       <c r="A90" s="1">
@@ -3833,6 +3875,12 @@
       <c r="E90">
         <v>87</v>
       </c>
+      <c r="F90" s="7">
+        <v>54773167.329999998</v>
+      </c>
+      <c r="G90">
+        <v>21288002</v>
+      </c>
     </row>
     <row r="91" spans="1:10" ht="18" x14ac:dyDescent="0.2">
       <c r="A91" s="1">
@@ -3850,6 +3898,12 @@
       <c r="E91">
         <v>202</v>
       </c>
+      <c r="F91" s="7">
+        <v>81000519.719999999</v>
+      </c>
+      <c r="G91">
+        <v>21251430</v>
+      </c>
     </row>
     <row r="92" spans="1:10" ht="18" x14ac:dyDescent="0.2">
       <c r="A92" s="1">
@@ -3867,6 +3921,12 @@
       <c r="E92">
         <v>288</v>
       </c>
+      <c r="F92" s="7">
+        <v>76771185.040000007</v>
+      </c>
+      <c r="G92">
+        <v>21226117</v>
+      </c>
     </row>
     <row r="93" spans="1:10" ht="18" x14ac:dyDescent="0.2">
       <c r="A93" s="1">
@@ -3884,6 +3944,12 @@
       <c r="E93">
         <v>253</v>
       </c>
+      <c r="F93" s="8">
+        <v>83357864.180000007</v>
+      </c>
+      <c r="G93">
+        <v>22023690</v>
+      </c>
     </row>
     <row r="94" spans="1:10" ht="18" x14ac:dyDescent="0.2">
       <c r="A94" s="1">
@@ -3901,6 +3967,12 @@
       <c r="E94">
         <v>94</v>
       </c>
+      <c r="F94" s="7">
+        <v>90146122.099999994</v>
+      </c>
+      <c r="G94">
+        <v>23253266</v>
+      </c>
     </row>
     <row r="95" spans="1:10" ht="18" x14ac:dyDescent="0.2">
       <c r="A95" s="1">
@@ -3918,6 +3990,12 @@
       <c r="E95">
         <v>6</v>
       </c>
+      <c r="F95" s="7">
+        <v>85283258.599999994</v>
+      </c>
+      <c r="G95">
+        <v>23979377</v>
+      </c>
     </row>
     <row r="96" spans="1:10" ht="18" x14ac:dyDescent="0.2">
       <c r="A96" s="1">
@@ -3935,6 +4013,12 @@
       <c r="E96">
         <v>0</v>
       </c>
+      <c r="F96" s="7">
+        <v>86488787.290000007</v>
+      </c>
+      <c r="G96">
+        <v>20715294</v>
+      </c>
     </row>
     <row r="97" spans="1:20" ht="18" x14ac:dyDescent="0.2">
       <c r="A97" s="1">
@@ -3952,6 +4036,12 @@
       <c r="E97">
         <v>0</v>
       </c>
+      <c r="F97" s="7">
+        <v>87661170.069999993</v>
+      </c>
+      <c r="G97">
+        <v>18880544</v>
+      </c>
     </row>
     <row r="98" spans="1:20" ht="18" x14ac:dyDescent="0.2">
       <c r="A98" s="1">
@@ -3969,6 +4059,12 @@
       <c r="E98">
         <v>0</v>
       </c>
+      <c r="F98" s="7">
+        <v>83441561.329999998</v>
+      </c>
+      <c r="G98">
+        <v>20017890</v>
+      </c>
     </row>
     <row r="99" spans="1:20" ht="18" x14ac:dyDescent="0.2">
       <c r="A99" s="1">
@@ -3986,6 +4082,12 @@
       <c r="E99">
         <v>0</v>
       </c>
+      <c r="F99" s="7">
+        <v>85863590.609999999</v>
+      </c>
+      <c r="G99">
+        <v>19539309</v>
+      </c>
     </row>
     <row r="100" spans="1:20" ht="18" x14ac:dyDescent="0.2">
       <c r="A100" s="1">
@@ -4002,6 +4104,12 @@
       </c>
       <c r="E100">
         <v>0</v>
+      </c>
+      <c r="F100" s="7">
+        <v>105284359.52</v>
+      </c>
+      <c r="G100">
+        <v>22580318</v>
       </c>
       <c r="H100" s="5"/>
       <c r="I100" s="5"/>
@@ -4031,6 +4139,12 @@
       </c>
       <c r="E101">
         <v>0</v>
+      </c>
+      <c r="F101" s="7">
+        <v>69640097.290000007</v>
+      </c>
+      <c r="G101">
+        <v>22499665</v>
       </c>
       <c r="H101" s="6"/>
       <c r="I101" s="5"/>
@@ -4062,6 +4176,12 @@
       <c r="E102">
         <v>62</v>
       </c>
+      <c r="F102" s="7">
+        <v>69001170.609999999</v>
+      </c>
+      <c r="G102">
+        <v>23980728</v>
+      </c>
       <c r="H102" s="6"/>
       <c r="I102" s="5"/>
       <c r="J102" s="5"/>
@@ -4092,6 +4212,12 @@
       <c r="E103">
         <v>159</v>
       </c>
+      <c r="F103" s="7">
+        <v>88051371.299999997</v>
+      </c>
+      <c r="G103">
+        <v>23436503</v>
+      </c>
       <c r="H103" s="5"/>
     </row>
     <row r="104" spans="1:20" ht="18" x14ac:dyDescent="0.2">
@@ -4109,6 +4235,12 @@
       </c>
       <c r="E104">
         <v>271</v>
+      </c>
+      <c r="F104" s="7">
+        <v>87385417.549999997</v>
+      </c>
+      <c r="G104">
+        <v>23370034</v>
       </c>
       <c r="H104" s="6"/>
       <c r="I104" s="5"/>
@@ -4140,6 +4272,12 @@
       <c r="E105">
         <v>236</v>
       </c>
+      <c r="F105" s="7">
+        <v>94717265.109999999</v>
+      </c>
+      <c r="G105">
+        <v>25378175</v>
+      </c>
     </row>
     <row r="106" spans="1:20" ht="18" x14ac:dyDescent="0.2">
       <c r="A106" s="1">
@@ -4157,6 +4295,12 @@
       <c r="E106">
         <v>107</v>
       </c>
+      <c r="F106" s="7">
+        <v>99929808.859999999</v>
+      </c>
+      <c r="G106">
+        <v>25931573</v>
+      </c>
     </row>
     <row r="107" spans="1:20" ht="18" x14ac:dyDescent="0.2">
       <c r="A107" s="1">
@@ -4174,6 +4318,12 @@
       <c r="E107">
         <v>11</v>
       </c>
+      <c r="F107" s="7">
+        <v>93508618.609999999</v>
+      </c>
+      <c r="G107">
+        <v>26871106</v>
+      </c>
     </row>
     <row r="108" spans="1:20" ht="18" x14ac:dyDescent="0.2">
       <c r="A108" s="1">
@@ -4191,6 +4341,12 @@
       <c r="E108">
         <v>0</v>
       </c>
+      <c r="F108" s="7">
+        <v>91728883.170000002</v>
+      </c>
+      <c r="G108">
+        <v>23595469</v>
+      </c>
     </row>
     <row r="109" spans="1:20" ht="18" x14ac:dyDescent="0.2">
       <c r="A109" s="1">
@@ -4208,6 +4364,12 @@
       <c r="E109">
         <v>0</v>
       </c>
+      <c r="F109" s="7">
+        <v>94242875.420000002</v>
+      </c>
+      <c r="G109">
+        <v>22503842</v>
+      </c>
     </row>
     <row r="110" spans="1:20" ht="18" x14ac:dyDescent="0.2">
       <c r="A110" s="1">
@@ -4225,6 +4387,12 @@
       <c r="E110">
         <v>0</v>
       </c>
+      <c r="F110" s="7">
+        <v>93362452.159999996</v>
+      </c>
+      <c r="G110">
+        <v>21162627</v>
+      </c>
     </row>
     <row r="111" spans="1:20" ht="18" x14ac:dyDescent="0.2">
       <c r="A111" s="1">
@@ -4242,6 +4410,12 @@
       <c r="E111">
         <v>0</v>
       </c>
+      <c r="F111" s="7">
+        <v>92005854.980000004</v>
+      </c>
+      <c r="G111">
+        <v>22980764</v>
+      </c>
     </row>
     <row r="112" spans="1:20" ht="18" x14ac:dyDescent="0.2">
       <c r="A112" s="1">
@@ -4259,8 +4433,14 @@
       <c r="E112">
         <v>0</v>
       </c>
-    </row>
-    <row r="113" spans="1:5" ht="18" x14ac:dyDescent="0.2">
+      <c r="F112" s="7">
+        <v>107555352.03</v>
+      </c>
+      <c r="G112">
+        <v>25289346</v>
+      </c>
+    </row>
+    <row r="113" spans="1:7" ht="18" x14ac:dyDescent="0.2">
       <c r="A113" s="1">
         <v>45383</v>
       </c>
@@ -4276,8 +4456,14 @@
       <c r="E113">
         <v>0</v>
       </c>
-    </row>
-    <row r="114" spans="1:5" ht="18" x14ac:dyDescent="0.2">
+      <c r="F113" s="7">
+        <v>77619361.969999999</v>
+      </c>
+      <c r="G113">
+        <v>25859186</v>
+      </c>
+    </row>
+    <row r="114" spans="1:7" ht="18" x14ac:dyDescent="0.2">
       <c r="A114" s="1">
         <v>45413</v>
       </c>
@@ -4293,8 +4479,14 @@
       <c r="E114">
         <v>102</v>
       </c>
-    </row>
-    <row r="115" spans="1:5" ht="18" x14ac:dyDescent="0.2">
+      <c r="F114" s="7">
+        <v>76173811.939999998</v>
+      </c>
+      <c r="G114">
+        <v>27376367</v>
+      </c>
+    </row>
+    <row r="115" spans="1:7" ht="18" x14ac:dyDescent="0.2">
       <c r="A115" s="1">
         <v>45444</v>
       </c>
@@ -4310,8 +4502,14 @@
       <c r="E115">
         <v>245</v>
       </c>
-    </row>
-    <row r="116" spans="1:5" ht="18" x14ac:dyDescent="0.2">
+      <c r="F115" s="7">
+        <v>89571094.930000007</v>
+      </c>
+      <c r="G115">
+        <v>26101791</v>
+      </c>
+    </row>
+    <row r="116" spans="1:7" ht="18" x14ac:dyDescent="0.2">
       <c r="A116" s="1">
         <v>45474</v>
       </c>
@@ -4327,8 +4525,14 @@
       <c r="E116">
         <v>262</v>
       </c>
-    </row>
-    <row r="117" spans="1:5" ht="18" x14ac:dyDescent="0.2">
+      <c r="F116" s="7">
+        <v>88354986.090000004</v>
+      </c>
+      <c r="G116">
+        <v>26356013</v>
+      </c>
+    </row>
+    <row r="117" spans="1:7" ht="18" x14ac:dyDescent="0.2">
       <c r="A117" s="1">
         <v>45505</v>
       </c>
@@ -4344,8 +4548,14 @@
       <c r="E117">
         <v>260</v>
       </c>
-    </row>
-    <row r="118" spans="1:5" ht="18" x14ac:dyDescent="0.2">
+      <c r="F117" s="7">
+        <v>97204929.780000001</v>
+      </c>
+      <c r="G117">
+        <v>27238227</v>
+      </c>
+    </row>
+    <row r="118" spans="1:7" ht="18" x14ac:dyDescent="0.2">
       <c r="A118" s="1">
         <v>45536</v>
       </c>
@@ -4361,8 +4571,14 @@
       <c r="E118">
         <v>142</v>
       </c>
-    </row>
-    <row r="119" spans="1:5" ht="18" x14ac:dyDescent="0.2">
+      <c r="F118" s="7">
+        <v>101434140.94</v>
+      </c>
+      <c r="G118">
+        <v>28092852</v>
+      </c>
+    </row>
+    <row r="119" spans="1:7" ht="18" x14ac:dyDescent="0.2">
       <c r="A119" s="1">
         <v>45566</v>
       </c>
@@ -4378,8 +4594,14 @@
       <c r="E119">
         <v>25</v>
       </c>
-    </row>
-    <row r="120" spans="1:5" ht="18" x14ac:dyDescent="0.2">
+      <c r="F119" s="7">
+        <v>94955036.439999998</v>
+      </c>
+      <c r="G119">
+        <v>29811979</v>
+      </c>
+    </row>
+    <row r="120" spans="1:7" ht="18" x14ac:dyDescent="0.2">
       <c r="A120" s="1">
         <v>45597</v>
       </c>
@@ -4395,8 +4617,14 @@
       <c r="E120">
         <v>0</v>
       </c>
-    </row>
-    <row r="121" spans="1:5" ht="18" x14ac:dyDescent="0.2">
+      <c r="F120" s="7">
+        <v>98916368.519999996</v>
+      </c>
+      <c r="G120">
+        <v>25086912</v>
+      </c>
+    </row>
+    <row r="121" spans="1:7" ht="18" x14ac:dyDescent="0.2">
       <c r="A121" s="1">
         <v>45627</v>
       </c>
@@ -4412,8 +4640,14 @@
       <c r="E121">
         <v>0</v>
       </c>
-    </row>
-    <row r="122" spans="1:5" ht="18" x14ac:dyDescent="0.2">
+      <c r="F121" s="8">
+        <v>94430022.099999994</v>
+      </c>
+      <c r="G121">
+        <v>23036270</v>
+      </c>
+    </row>
+    <row r="122" spans="1:7" ht="18" x14ac:dyDescent="0.2">
       <c r="A122" s="1">
         <v>45658</v>
       </c>
@@ -4429,8 +4663,14 @@
       <c r="E122">
         <v>0</v>
       </c>
-    </row>
-    <row r="123" spans="1:5" ht="18" x14ac:dyDescent="0.2">
+      <c r="F122" s="7">
+        <v>92999053.799999997</v>
+      </c>
+      <c r="G122">
+        <v>23897201</v>
+      </c>
+    </row>
+    <row r="123" spans="1:7" ht="18" x14ac:dyDescent="0.2">
       <c r="A123" s="1">
         <v>45689</v>
       </c>
@@ -4446,8 +4686,14 @@
       <c r="E123">
         <v>0</v>
       </c>
-    </row>
-    <row r="124" spans="1:5" ht="18" x14ac:dyDescent="0.2">
+      <c r="F123" s="7">
+        <v>95935715.430000007</v>
+      </c>
+      <c r="G123">
+        <v>24037128</v>
+      </c>
+    </row>
+    <row r="124" spans="1:7" ht="18" x14ac:dyDescent="0.2">
       <c r="A124" s="1">
         <v>45717</v>
       </c>
@@ -4463,8 +4709,14 @@
       <c r="E124">
         <v>0</v>
       </c>
-    </row>
-    <row r="125" spans="1:5" ht="18" x14ac:dyDescent="0.2">
+      <c r="F124" s="7">
+        <v>108845450.02</v>
+      </c>
+      <c r="G124">
+        <v>28285212</v>
+      </c>
+    </row>
+    <row r="125" spans="1:7" ht="18" x14ac:dyDescent="0.2">
       <c r="A125" s="1">
         <v>45748</v>
       </c>
@@ -4480,8 +4732,14 @@
       <c r="E125">
         <v>0</v>
       </c>
-    </row>
-    <row r="126" spans="1:5" ht="18" x14ac:dyDescent="0.2">
+      <c r="F125" s="7">
+        <v>80837585.560000002</v>
+      </c>
+      <c r="G125">
+        <v>28849640</v>
+      </c>
+    </row>
+    <row r="126" spans="1:7" ht="18" x14ac:dyDescent="0.2">
       <c r="A126" s="1">
         <v>45778</v>
       </c>
@@ -4497,8 +4755,14 @@
       <c r="E126">
         <v>31</v>
       </c>
-    </row>
-    <row r="127" spans="1:5" ht="18" x14ac:dyDescent="0.2">
+      <c r="F126" s="7">
+        <v>80294648.319999993</v>
+      </c>
+      <c r="G126">
+        <v>29862445</v>
+      </c>
+    </row>
+    <row r="127" spans="1:7" ht="18" x14ac:dyDescent="0.2">
       <c r="A127" s="1">
         <v>45809</v>
       </c>
@@ -4514,8 +4778,14 @@
       <c r="E127">
         <v>237</v>
       </c>
-    </row>
-    <row r="128" spans="1:5" ht="18" x14ac:dyDescent="0.2">
+      <c r="F127" s="7">
+        <v>92492155.849999994</v>
+      </c>
+      <c r="G127">
+        <v>28962021</v>
+      </c>
+    </row>
+    <row r="128" spans="1:7" ht="18" x14ac:dyDescent="0.2">
       <c r="A128" s="1">
         <v>45839</v>
       </c>
@@ -4530,6 +4800,12 @@
       </c>
       <c r="E128">
         <v>357</v>
+      </c>
+      <c r="F128" s="7">
+        <v>89847351.170000002</v>
+      </c>
+      <c r="G128">
+        <v>29447751</v>
       </c>
     </row>
     <row r="129" spans="1:18" ht="18" x14ac:dyDescent="0.2">
@@ -4548,6 +4824,12 @@
       <c r="E129">
         <v>238</v>
       </c>
+      <c r="F129" s="7">
+        <v>101538463.09999999</v>
+      </c>
+      <c r="G129">
+        <v>31212871</v>
+      </c>
     </row>
     <row r="130" spans="1:18" ht="18" x14ac:dyDescent="0.2">
       <c r="A130" s="1">
@@ -4565,6 +4847,12 @@
       <c r="E130">
         <v>120</v>
       </c>
+      <c r="F130" s="7">
+        <v>101843015.98999999</v>
+      </c>
+      <c r="G130">
+        <v>30630011</v>
+      </c>
     </row>
     <row r="131" spans="1:18" ht="18" x14ac:dyDescent="0.2">
       <c r="A131" s="1">
@@ -4582,6 +4870,12 @@
       <c r="E131">
         <v>19</v>
       </c>
+      <c r="F131" s="7">
+        <v>97796697.25</v>
+      </c>
+      <c r="G131">
+        <v>31647401</v>
+      </c>
     </row>
     <row r="132" spans="1:18" ht="18" x14ac:dyDescent="0.2">
       <c r="A132" s="1">
@@ -4598,6 +4892,12 @@
       </c>
       <c r="E132">
         <v>0</v>
+      </c>
+      <c r="F132" s="7">
+        <v>100002404.53</v>
+      </c>
+      <c r="G132">
+        <v>26800473</v>
       </c>
       <c r="K132" s="5"/>
       <c r="L132" s="5"/>
@@ -4624,6 +4924,12 @@
       <c r="E133">
         <v>0</v>
       </c>
+      <c r="F133" s="7">
+        <v>102228337.48999999</v>
+      </c>
+      <c r="G133">
+        <v>24587033</v>
+      </c>
     </row>
     <row r="134" spans="1:18" ht="18" x14ac:dyDescent="0.2">
       <c r="A134" s="1">
@@ -4641,6 +4947,12 @@
       <c r="E134">
         <v>0</v>
       </c>
+      <c r="F134" s="8">
+        <v>109324242.63</v>
+      </c>
+      <c r="G134">
+        <v>24436679</v>
+      </c>
     </row>
     <row r="135" spans="1:18" ht="18" x14ac:dyDescent="0.2">
       <c r="A135" s="1">
@@ -4658,6 +4970,12 @@
       <c r="E135">
         <v>0</v>
       </c>
+      <c r="F135" s="7">
+        <v>99158732.650000006</v>
+      </c>
+      <c r="G135">
+        <v>25560991</v>
+      </c>
     </row>
     <row r="136" spans="1:18" ht="18" x14ac:dyDescent="0.2">
       <c r="A136" s="1">
@@ -4675,6 +4993,12 @@
       <c r="E136">
         <v>0</v>
       </c>
+      <c r="F136" s="7">
+        <v>116815151.63</v>
+      </c>
+      <c r="G136">
+        <v>28624796</v>
+      </c>
     </row>
     <row r="137" spans="1:18" ht="18" x14ac:dyDescent="0.2">
       <c r="A137" s="1">
@@ -4691,6 +5015,12 @@
       </c>
       <c r="E137">
         <v>6</v>
+      </c>
+      <c r="F137" s="7">
+        <v>94531070.400000006</v>
+      </c>
+      <c r="G137">
+        <v>29366823</v>
       </c>
     </row>
     <row r="138" spans="1:18" x14ac:dyDescent="0.2">

</xml_diff>